<commit_message>
V12: add drug-label comparison (SIDER 4.1), READUS-PV checklist, AI disclosure, GCNMLP comparison table
</commit_message>
<xml_diff>
--- a/Supplementary_Information/S1_Table_STROBE_Checklist.xlsx
+++ b/Supplementary_Information/S1_Table_STROBE_Checklist.xlsx
@@ -597,7 +597,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Introduction, final two paragraphs: aims of PulseTech and the three stated results</t>
+          <t>Introduction, final two paragraphs: aims of PulseTech and the four stated results</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Methods - Classical disproportionality analysis: drug-ADR pairs (MedDRA Preferred Terms as coded in FAERS), 2x2 contingency table, PRR, ROR, IC and EBGM (Eqs 1-2); S5 Table</t>
+          <t>Methods - Classical disproportionality analysis: drugs in the primary-suspect role; drug-ADR pairs (MedDRA Preferred Terms as coded in FAERS), 2x2 contingency table, PRR, ROR, IC and EBGM (Eqs 1-2); S5 Table</t>
         </is>
       </c>
     </row>
@@ -739,7 +739,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Table 4 Steps 2 (case deduplication), 4 (unresolved age retained to avoid denominator bias) and 8 (restriction to pediatric records); Discussion - Threats to validity and Limitations</t>
+          <t>Table 4 Steps 2 (case deduplication), 4 (unresolved age retained to avoid denominator bias) and 8 (restriction to pediatric records); Methods - Comparison with drug labels (indication, product-use and exposure term categories, S9 Table); Discussion - Threats to validity and Limitations</t>
         </is>
       </c>
     </row>
@@ -805,7 +805,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Methods - Classical disproportionality analysis (Eqs 1-2) and The PulseTech HANConv architecture (Eqs 3-7, Table 5)</t>
+          <t>Methods - Classical disproportionality analysis (Eqs 1-2), Comparison with drug labels (SIDER 4.1, MedDRA 28.1 term categories, AUC; S9 Table) and The PulseTech HANConv architecture (Eqs 3-7, Table 5)</t>
         </is>
       </c>
     </row>
@@ -925,7 +925,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Results - Top drug-ADR co-occurrences (Table 11); Link-prediction performance (Table 12); Candidate drug-ADR links: a worked illustration (Table 13); Recent-quarter trend analysis</t>
+          <t>Results - Comparison with drug labels (S9 Table); Top drug-ADR co-occurrences (Table 11); Link-prediction performance (Table 12); Candidate drug-ADR links: a worked illustration (Table 13); Recent-quarter trend analysis</t>
         </is>
       </c>
     </row>

</xml_diff>